<commit_message>
updates with phylogeny analysis
</commit_message>
<xml_diff>
--- a/results/expected_output/cohort_metadata_summary.xlsx
+++ b/results/expected_output/cohort_metadata_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,29 +506,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SRR25276878</t>
+          <t>ERR11759336</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SAMN36448984</t>
+          <t>SAMEA114110082</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2022-10-20</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>MNH_G2C5F</t>
-        </is>
-      </c>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>SRA_PE</t>
@@ -538,13 +534,13 @@
         <v>98.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>85.89</v>
+        <v>91.2</v>
       </c>
       <c r="I2" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
-        <v>5390038</v>
+        <v>5392788</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>
@@ -569,12 +565,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SRR38361580</t>
+          <t>ERR11759339</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SAMN57562819</t>
+          <t>SAMEA114110085</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -584,7 +580,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -597,13 +593,13 @@
         <v>98.59999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>81.18000000000001</v>
+        <v>392.1</v>
       </c>
       <c r="I3" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="J3" t="n">
-        <v>5518281</v>
+        <v>5373271</v>
       </c>
       <c r="K3" t="b">
         <v>1</v>
@@ -616,17 +612,513 @@
       <c r="M3" t="b">
         <v>1</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="Q3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ERR11759340</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SAMEA114110086</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="H4" t="n">
+        <v>307.72</v>
+      </c>
+      <c r="I4" t="n">
+        <v>56</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5401290</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ERR11759341</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SAMEA114110087</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>96.56999999999999</v>
+      </c>
+      <c r="I5" t="n">
         <v>100</v>
       </c>
-      <c r="O3" t="b">
-        <v>1</v>
-      </c>
-      <c r="P3" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q3" t="b">
-        <v>1</v>
+      <c r="J5" t="n">
+        <v>5226013</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ERR11759342</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SAMEA114110088</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>115.34</v>
+      </c>
+      <c r="I6" t="n">
+        <v>82</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5561800</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ERR11759343</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SAMEA114110089</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="H7" t="n">
+        <v>308.78</v>
+      </c>
+      <c r="I7" t="n">
+        <v>95</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5419236</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="b">
+        <v>0</v>
+      </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ERR11759344</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SAMEA114110090</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="H8" t="n">
+        <v>250</v>
+      </c>
+      <c r="I8" t="n">
+        <v>54</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5531550</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="O8" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="Q8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ERR11759345</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SAMEA114110091</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="H9" t="n">
+        <v>89.63</v>
+      </c>
+      <c r="I9" t="n">
+        <v>67</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5195552</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="b">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SRR4423335</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SAMN05908511</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2015-06</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DA48896</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>56.33</v>
+      </c>
+      <c r="I10" t="n">
+        <v>110</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5642446</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="O10" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="Q10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ERR5685495</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SAMEA8515318</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2015-17</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SRA_PE</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="H11" t="n">
+        <v>44.21</v>
+      </c>
+      <c r="I11" t="n">
+        <v>182</v>
+      </c>
+      <c r="J11" t="n">
+        <v>5804927</v>
+      </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Coverage 44.21x &lt; 50.0x</t>
+        </is>
+      </c>
+      <c r="M11" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="b">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>